<commit_message>
modify apis, api4 todo
</commit_message>
<xml_diff>
--- a/Risk2SQL/data/SourceData.xlsx
+++ b/Risk2SQL/data/SourceData.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="96">
   <si>
     <t>序列</t>
   </si>
@@ -87,12 +87,6 @@
     <t>提供审计问题库信息</t>
   </si>
   <si>
-    <t>国网运检部关于印发电网生产设备分类和固定资产目录对应关系的通知(运检计划〔2013〕547号)</t>
-  </si>
-  <si>
-    <t>提供建账建卡规范性要求</t>
-  </si>
-  <si>
     <t>系统</t>
   </si>
   <si>
@@ -124,6 +118,7 @@
   </si>
   <si>
     <t>PSPID-项目编码
+,pro_year-项目年份
     ,POST1-描述
     ,PRCTR-利润中心
     ,VBUKR-公司代码
@@ -167,7 +162,7 @@
     ,value_old-旧值</t>
   </si>
   <si>
-    <t>表：BSEG\BKPF</t>
+    <t>表：BSEG/BKPF</t>
   </si>
   <si>
     <t>项目编码PSPID、单体工程号POSID、、转资凭证中的凭证日期BLDAT</t>
@@ -215,22 +210,140 @@
     <t>数据中台</t>
   </si>
   <si>
-    <t>表：pro_swid01_prd.dws_ast_zcqsm_wzsj_cgsq_info_mf</t>
+    <t>表：dws_ast_as_wzsj_cgsq_info_df</t>
   </si>
   <si>
     <t>提供项目关联的采购申请信息</t>
   </si>
   <si>
-    <t>dws_ast_zcqsm_wzsj_cgsq_info_mf</t>
-  </si>
-  <si>
-    <t>表：pro_swid01_prd.dws_ast_zcqsm_wzsj_cgdd_info_mf</t>
+    <t>dws_ast_as_wzsj_cgsq_info_df</t>
+  </si>
+  <si>
+    <t>pspid-项目编码
+    ,posid-单体工程编码
+    ,mandt-客户端
+    ,scbs_cgsq-删除标识
+    ,yxbs-有效标识
+    ,cgsq-采购申请
+    ,hxm_cgsq-行项目
+    ,cgms-采购描述
+    ,wlb-物料编码
+    ,wlms-物料描述
+    ,fwbh-服务编号
+    ,fwbhms-服务编号描述
+    ,wlz-物料组
+    ,wlzms-物料组描述
+    ,cgxzb-采购性质编码
+    ,cgxzms-采购性质描述
+    ,pzlx_cgsq-凭证类型
+    ,pzlxmc-凭证类型名称
+    ,pzbs_cgsq-批准标识
+    ,pzbsms-批准标识描述
+    ,cjz-创建者
+    ,cjzx-创建者姓名
+    ,ssdq-所属地区
+    ,gcb-工厂编码
+    ,gcms-工厂描述
+    ,cgzz-采购组织
+    ,cgzzms-采购组织描述
+    ,cgz-采购组
+    ,cgzms-采购组描述
+    ,sqsl-申请数量
+    ,jldw-计量单位
+    ,sqdj-申请单价
+    ,jgdw-价格单位
+    ,sqzj-申请总价（审批后）
+    ,jsgfsid-技术规范书ID
+    ,cgpcb-采购批次编码
+    ,cgpcmc-采购批次名称
+    ,zsgcgpc-首个采购批次
+    ,kjxy-框架协议
+    ,hxm_kjxy-行项目
+    ,glbs-关联标识:1补充关联 0:正常关联
+    ,cgdd-采购订单
+    ,hxm_cgdd-行项目
+    ,scbs_cgdd-删除标识
+    ,qgdh_ds-请购单号（电商采购专区）
+    ,hxm_qgdh_ds-行项目
+    ,qgdh_ksh-请购单号（可视化选购专区）
+    ,hxm_qgdh_ksh-行项目
+    ,wsqgd-网商请购单
+    ,wbs-WBS元素
+    ,wbsms-WBS描述
+    ,xmmc-项目名称
+    ,wbs_dt-WBS元素（单体）
+    ,wbsms_dt-WBS描述（单体）
+    ,cjrq-创建日期
+    ,jhrq-交货日期
+    ,pzrq-批准日期</t>
+  </si>
+  <si>
+    <t>表：dws_ast_as_wzsj_cgdd_info_df</t>
   </si>
   <si>
     <t>提供项目关联的采购订单信息</t>
   </si>
   <si>
-    <t>dws_ast_zcqsm_wzsj_cgdd_info_mf</t>
+    <t>dws_ast_as_wzsj_cgdd_info_df</t>
+  </si>
+  <si>
+    <t>pspid-项目编码
+    ,posid-单体工程编码
+    ,mandt-客户端
+    ,scbs_cgdd-删除标识
+    ,cgdd-采购订单
+    ,hxm_cgdd-行项目
+    ,cgddms-采购订单描述
+    ,wlbm-物料编码
+    ,wlms-物料描述
+    ,fwbh-服务编号
+    ,fwbhms-服务编号描述
+    ,wlz-物料组
+    ,wlzms-物料组描述
+    ,dds-订单数量
+    ,jldw-计量单位
+    ,ddjj-订单净价
+    ,ddzj-订单总价
+    ,jgdw-价格单位
+    ,wbs-WBS元素
+    ,wbsms-WBS描述
+    ,xmms-项目描述
+    ,gsdm-公司代码
+    ,gsms-公司描述
+    ,ssdq-所属地区
+    ,gcbm-工厂编码
+    ,gcms-工厂描述
+    ,kcdd-库存地点
+    ,kcddms-库存地点描述
+    ,cgsq-采购申请
+    ,hxm_cgsq-行项目
+    ,htbh-合同编号
+    ,hxm_htbh-行项目
+    ,jhrq-交货日期
+    ,dhrq-到货日期
+    ,dhje-到货金额
+    ,ckrq-出库日期
+    ,pzlx_cgdd-凭证类型
+    ,pzlxms-凭证类型描述
+    ,pzbs_cgdd-批准标识
+    ,pzbsms-批准标识描述
+    ,pzrq-凭证日期
+    ,cjrq-创建日期
+    ,cjz-创建者
+    ,cjzxm-创建者姓名
+    ,gys-供应商
+    ,gysms-供应商描述
+    ,cgzz-采购组织
+    ,cgzzms-采购组织描述
+    ,cgz-采购组
+    ,cgzms-采购组描述
+    ,ddzjz-订单总计值（下达时）
+    ,gysxz-供应商性质
+    ,sgf-施工费
+    ,sjf-设计费
+    ,jlf-监理费
+    ,zjzxf-造价咨询费
+    ,fwqrje-服务确认金额</t>
   </si>
   <si>
     <t>表：MSEG/MKPF</t>
@@ -302,7 +415,26 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>(415Q)</t>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>415</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)、特殊库存标识sobkz（Q）</t>
     </r>
     <r>
       <rPr>
@@ -1151,6 +1283,11 @@
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="00FF0000"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1409,11 +1546,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="3"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="7" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="13" style="8" customWidth="1"/>
-    <col min="2" max="2" width="96.1818181818182" customWidth="1"/>
+    <col min="2" max="2" width="54.1090909090909" customWidth="1"/>
     <col min="3" max="3" width="11.3545454545455" customWidth="1"/>
     <col min="4" max="4" width="38.5454545454545" customWidth="1"/>
   </cols>
@@ -1522,20 +1659,6 @@
       </c>
       <c r="D8" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="8">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1553,8 +1676,8 @@
   <cols>
     <col min="1" max="1" width="5.81818181818182" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.1818181818182" style="1" customWidth="1"/>
-    <col min="3" max="3" width="46.6363636363636" style="2" customWidth="1"/>
-    <col min="4" max="4" width="53.6454545454545" style="2" customWidth="1"/>
+    <col min="3" max="3" width="25.8909090909091" style="2" customWidth="1"/>
+    <col min="4" max="4" width="53.6363636363636" style="2" customWidth="1"/>
     <col min="5" max="5" width="41.8909090909091" style="2" customWidth="1"/>
     <col min="6" max="6" width="15.5545454545455" style="2" customWidth="1"/>
     <col min="7" max="7" width="16.1090909090909" style="2" customWidth="1"/>
@@ -1568,74 +1691,74 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>21</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>23</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" ht="252" spans="1:9">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" ht="266" spans="1:9">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="G2" s="2">
         <v>1</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" ht="252" spans="1:9">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" ht="266" spans="1:9">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="G3" s="2">
         <v>1</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:9">
@@ -1643,25 +1766,25 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="G4" s="2">
         <v>2</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:9">
@@ -1669,25 +1792,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="G5" s="2">
         <v>3</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" ht="224" spans="1:9">
@@ -1695,58 +1818,64 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>47</v>
       </c>
       <c r="G6" s="2">
         <v>14</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" ht="28" spans="1:8">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" ht="409.5" spans="1:9">
       <c r="A7" s="1">
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="I7" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1" spans="1:8">
+    </row>
+    <row r="8" ht="45" customHeight="1" spans="1:9">
       <c r="A8" s="1">
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="I8" s="7" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1755,7 +1884,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>57</v>
@@ -1778,7 +1907,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>61</v>
@@ -1801,7 +1930,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>57</v>
@@ -1819,12 +1948,12 @@
         <v>67</v>
       </c>
     </row>
-    <row r="12" ht="52" customHeight="1" spans="1:8">
+    <row r="12" spans="1:8">
       <c r="A12" s="1">
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>68</v>
@@ -1856,12 +1985,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" ht="252" spans="1:9">
+    <row r="14" ht="266" spans="1:9">
       <c r="A14" s="1">
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>73</v>
@@ -1876,10 +2005,10 @@
         <v>1</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" ht="140" spans="1:9">
@@ -1887,7 +2016,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>76</v>
@@ -1913,7 +2042,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>81</v>
@@ -1939,7 +2068,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>86</v>
@@ -1965,7 +2094,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>91</v>

</xml_diff>